<commit_message>
feat(admin): roll out 2FA security hardening and console UX upgrades
</commit_message>
<xml_diff>
--- a/output/spreadsheet/startpray-progress-tracker.xlsx
+++ b/output/spreadsheet/startpray-progress-tracker.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>c85c8b0</t>
+          <t>9d00e9c</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-03-15 14:21:40</t>
+          <t>2026-03-21 17:40:55</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3606,14 +3606,80 @@
           <t>[AUTO] Manual sync: main @ c85c8b0</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>Update task status and release mapping.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-03-21 15:20:22</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ ea30eb9</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-03-21 15:53:04</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ 9ac4d0b</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-03-21 17:40:55</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ 9d00e9c</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
         <is>
           <t>git-hook</t>
         </is>
@@ -3754,7 +3820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4183,7 +4249,118 @@
           <t>https://github.com/dan40912/prayer-coin.git</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-03-21 15:20:22</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ea30eb9</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>(no tag)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>chore: sync latest portal, player, and home updates</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/prayer-coin.git</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-03-21 15:53:04</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>9ac4d0b</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>(no tag)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>fix: restore logo path and harden prayer audio playback</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/prayer-coin.git</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-03-21 17:40:55</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>9d00e9c</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>(no tag)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>fix: stabilize prayfor audio and mobile header/player UI</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/prayer-coin.git</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: improve SEO metadata, footer spacing, and customer image upload flow
- Add/refresh page metadata across public routes, including dynamic prayfor detail metadata format.

- Remove extra footer-bottom whitespace by applying body padding only when global player is mounted.

- Harden customer create image flow: remove external cover URL input, require internal /uploads assets, raise upload cap to 10MB.

- Enforce backend validation for image/gallery URLs and restore sanitized payload handling for home-card creation.

- Update upload API to always compress and store images as webp for consistent storage output.

- Add remote 2FA deployment guide and route-level metadata layouts for auth/customer portal pages.
</commit_message>
<xml_diff>
--- a/output/spreadsheet/startpray-progress-tracker.xlsx
+++ b/output/spreadsheet/startpray-progress-tracker.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>9d00e9c</t>
+          <t>d320697</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21 17:40:55</t>
+          <t>2026-03-24 23:37:09</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3672,14 +3672,36 @@
           <t>[AUTO] Commit recorded: main @ 9d00e9c</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>Continue task updates and prepare push.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-03-24 23:37:09</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ d320697</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
         <is>
           <t>git-hook</t>
         </is>
@@ -3820,7 +3842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4360,7 +4382,44 @@
           <t>https://github.com/dan40912/prayer-coin.git</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-03-24 23:37:09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>d320697</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>(no tag)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>feat(admin): roll out 2FA security hardening and console UX upgrades</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/prayer-coin.git</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: finalize admin editors/player updates and add prod migration bundle
</commit_message>
<xml_diff>
--- a/output/spreadsheet/startpray-progress-tracker.xlsx
+++ b/output/spreadsheet/startpray-progress-tracker.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-23148" yWindow="-2616" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,35 +18,87 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$M$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Release_Tracker'!$A$1:$J$2</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="11">
     <font>
-      <name val="Calibri"/>
+      <name val="新細明體"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="新細明體"/>
+      <charset val="136"/>
+      <family val="1"/>
       <b val="1"/>
       <sz val="16"/>
     </font>
     <font>
+      <name val="新細明體"/>
+      <charset val="136"/>
+      <family val="1"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="新細明體"/>
+      <charset val="136"/>
+      <family val="1"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="新細明體"/>
+      <charset val="136"/>
+      <family val="1"/>
       <b val="1"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <color rgb="FF0D0D0D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF0D0D0D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <color rgb="FF0D0D0D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <family val="3"/>
+      <color rgb="FF0D0D0D"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <family val="3"/>
+      <color rgb="FF0285FF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="新細明體"/>
+      <charset val="136"/>
+      <family val="3"/>
+      <sz val="9"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -59,12 +110,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EAF2F8"/>
+        <fgColor rgb="FFEAF2F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -78,23 +129,24 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -107,9 +159,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -472,8 +539,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:G60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -483,7 +550,7 @@
     <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Start Pray ??????</t>
@@ -532,7 +599,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>d320697</t>
+          <t>367b31a</t>
         </is>
       </c>
     </row>
@@ -574,7 +641,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-03-24 23:37:09</t>
+          <t>2026-03-28 21:35:01</t>
         </is>
       </c>
     </row>
@@ -823,6 +890,251 @@
       <c r="D21" s="8">
         <f>IFERROR(C21/B21,0)</f>
         <v/>
+      </c>
+    </row>
+    <row r="26" ht="28.5" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>前台優先小修版改造 + 安全/架構優化路線圖</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="71.25" customHeight="1">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>你選擇的策略：先做前台體驗、第一階段只做小修補、後台先下架未完成頁，同時要清楚列出安全與架構優化路線。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="28.5" customHeight="1">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>盤點後的高風險不合理點（需納入路線）：</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="42.75" customHeight="1">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>1. 客戶端可偽造登入身分（auth-storage.js、server-session.js）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="95.25" customHeight="1">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>2. 公開 API 存在敏感資料外洩/越權風險（api/users/route.js、api/responses/[homeCardId]/route.js、api/home-cards/route.js）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="71.25" customHeight="1">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>3. 前台樣式層過度膨脹與重疊（globals.css 約 7.6k 行，主題檔重複定義），影響美觀一致性與維護。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="71.25" customHeight="1">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>4. 後台資訊架構混雜真/假頁面（analytics/finance/moderation/support 為 mock），降低管理可信度。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="69" customHeight="1">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>5. API 存在舊版殘留與失配（/api/prayers*、/api/PrayerResponse、/api/home-cards/[id]）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>Implementation Changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="28.5" customHeight="1">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>第一階段（前台小修補，2-3 週，先做）</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="57" customHeight="1">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>1. 視覺一致性小修：統一首頁、祈禱牆、詳情頁的字級、留白、按鈕層級與卡片密度，不重做版型。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="57" customHeight="1">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>2. 內容豐富化小修：補強首頁「信任感區塊」與「引導區塊」文案層次，優化空狀態與錯誤提示。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="57" customHeight="1">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>3. 互動精修：減少首頁探索區過重的即時請求（保留功能但降載），優化載入中/無結果體驗。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="42.75" customHeight="1">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>4. 後台導航清理：先隱藏未完成 mock 模組，只保留已串接可運作頁面。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="42.75" customHeight="1">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>第二階段（安全與架構優化路線，並行設計、下階段落地）</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="85.5" customHeight="1">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>5. Session 重構：改為 server 簽章/驗證 session（httpOnly），移除對可竄改 client cookie/localStorage 的信任。</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="99.75" customHeight="1">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>6. Public API 收斂：下架或封鎖高風險舊 API（/api/users、/api/prayers*、/api/PrayerResponse），補上最小必要欄位 select。</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="85.5" customHeight="1">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>7. 權限與資料流一致化：home-cards/responses 建立與修改改為 server 端用 session 決定 ownerId/responderId，不再吃前端傳入 ID。</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="85.5" customHeight="1">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>8. Admin 邏輯一致化：每支 admin route 補顯式權限檢查（非僅依賴 middleware header），整理 banner 為單一資料來源。</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="28.5" customHeight="1">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>介面/API 變更（先規劃）</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="40.5" customHeight="1">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>9. POST /api/home-cards：移除 ownerId 請求欄位，由 server 注入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="54.75" customHeight="1">
+      <c r="A48" s="14" t="inlineStr">
+        <is>
+          <t>10. POST /api/responses：移除 responderId 請求欄位，由 server 注入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="81" customHeight="1">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>11. /api/responses/[homeCardId]：回傳 responder 白名單欄位（name/avatar），不回傳完整 user model。</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="71.25" customHeight="1">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t>12. /api/users、/api/prayers*、/api/PrayerResponse：標記淘汰並移除外部可用性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>Test Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="57" customHeight="1">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
+          <t>1. 前台回歸：首頁、祈禱牆、詳情、登入/註冊、會員中心在 desktop/mobile 版面與互動檢查。</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="71.25" customHeight="1">
+      <c r="A53" s="12" t="inlineStr">
+        <is>
+          <t>2. 安全驗證：手動竄改 pc-auth cookie/localStorage 後，不可讀寫他人資料；未登入不可建立卡片/回應。</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="57" customHeight="1">
+      <c r="A54" s="12" t="inlineStr">
+        <is>
+          <t>3. API 合約：建立/查詢/檢舉/後台封鎖流程的成功與拒絕案例（401/403/422）要明確。</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="57" customHeight="1">
+      <c r="A55" s="12" t="inlineStr">
+        <is>
+          <t>4. 建置品質：npm run lint、npm run build 必須無新增警告與無路由失配。</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="11" t="inlineStr">
+        <is>
+          <t>Assumptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="42.75" customHeight="1">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t>1. 第一階段不做全面重設計，只做「高感知小修補」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="42.75" customHeight="1">
+      <c r="A58" s="12" t="inlineStr">
+        <is>
+          <t>2. 後台未完成頁面先隱藏，不在第一階段補齊全部功能。</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="42.75" customHeight="1">
+      <c r="A59" s="12" t="inlineStr">
+        <is>
+          <t>3. 安全與架構路線本輪先定規格與優先級，實作安排在下一階段。</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="42.75" customHeight="1">
+      <c r="A60" s="12" t="inlineStr">
+        <is>
+          <t>4. 不變更品牌核心定位與主要內容語言（維持現有中文主體）。</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -837,13 +1149,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="4" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
@@ -920,7 +1231,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="31.5" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
           <t>UX-02</t>
@@ -1025,7 +1336,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="31.5" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>UX-05</t>
@@ -1095,7 +1406,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="31.5" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
           <t>UX-07</t>
@@ -1130,7 +1441,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="31.5" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
           <t>UX-08</t>
@@ -1178,10 +1489,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M40"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -1191,8 +1501,7 @@
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="12" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1262,7 +1571,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="31.5" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>TASK-001</t>
@@ -1291,8 +1600,8 @@
       <c r="F2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="9" t="inlineStr"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="9" t="n"/>
       <c r="I2" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -1303,9 +1612,9 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K2" s="9" t="inlineStr"/>
-      <c r="L2" s="3" t="inlineStr"/>
-      <c r="M2" s="3" t="inlineStr"/>
+      <c r="K2" s="9" t="n"/>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1336,8 +1645,8 @@
       <c r="F3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="9" t="inlineStr"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="9" t="n"/>
       <c r="I3" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -1348,9 +1657,9 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K3" s="9" t="inlineStr"/>
-      <c r="L3" s="3" t="inlineStr"/>
-      <c r="M3" s="3" t="inlineStr"/>
+      <c r="K3" s="9" t="n"/>
+      <c r="L3" s="3" t="n"/>
+      <c r="M3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1381,8 +1690,8 @@
       <c r="F4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="9" t="inlineStr"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="9" t="n"/>
       <c r="I4" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -1393,11 +1702,11 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K4" s="9" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr"/>
-      <c r="M4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
+      <c r="K4" s="9" t="n"/>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="31.5" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>TASK-004</t>
@@ -1426,8 +1735,8 @@
       <c r="F5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="9" t="inlineStr"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="9" t="n"/>
       <c r="I5" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -1438,9 +1747,9 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K5" s="9" t="inlineStr"/>
-      <c r="L5" s="3" t="inlineStr"/>
-      <c r="M5" s="3" t="inlineStr"/>
+      <c r="K5" s="9" t="n"/>
+      <c r="L5" s="3" t="n"/>
+      <c r="M5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1471,8 +1780,8 @@
       <c r="F6" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="9" t="inlineStr"/>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="9" t="n"/>
       <c r="I6" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -1483,9 +1792,9 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K6" s="9" t="inlineStr"/>
-      <c r="L6" s="3" t="inlineStr"/>
-      <c r="M6" s="3" t="inlineStr"/>
+      <c r="K6" s="9" t="n"/>
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1516,8 +1825,8 @@
       <c r="F7" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="9" t="inlineStr"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="9" t="n"/>
       <c r="I7" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -1528,9 +1837,9 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K7" s="9" t="inlineStr"/>
-      <c r="L7" s="3" t="inlineStr"/>
-      <c r="M7" s="3" t="inlineStr"/>
+      <c r="K7" s="9" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1561,8 +1870,8 @@
       <c r="F8" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="9" t="inlineStr"/>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="9" t="n"/>
       <c r="I8" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -1573,9 +1882,9 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K8" s="9" t="inlineStr"/>
-      <c r="L8" s="3" t="inlineStr"/>
-      <c r="M8" s="3" t="inlineStr"/>
+      <c r="K8" s="9" t="n"/>
+      <c r="L8" s="3" t="n"/>
+      <c r="M8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1606,8 +1915,8 @@
       <c r="F9" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="9" t="inlineStr"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="9" t="n"/>
       <c r="I9" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -1618,9 +1927,9 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K9" s="9" t="inlineStr"/>
-      <c r="L9" s="3" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr"/>
+      <c r="K9" s="9" t="n"/>
+      <c r="L9" s="3" t="n"/>
+      <c r="M9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1651,8 +1960,8 @@
       <c r="F10" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="3" t="inlineStr"/>
-      <c r="H10" s="9" t="inlineStr"/>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="9" t="n"/>
       <c r="I10" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -1663,9 +1972,9 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K10" s="9" t="inlineStr"/>
-      <c r="L10" s="3" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr"/>
+      <c r="K10" s="9" t="n"/>
+      <c r="L10" s="3" t="n"/>
+      <c r="M10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1696,8 +2005,8 @@
       <c r="F11" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="9" t="inlineStr"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="9" t="n"/>
       <c r="I11" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -1708,11 +2017,11 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K11" s="9" t="inlineStr"/>
-      <c r="L11" s="3" t="inlineStr"/>
-      <c r="M11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
+      <c r="K11" s="9" t="n"/>
+      <c r="L11" s="3" t="n"/>
+      <c r="M11" s="3" t="n"/>
+    </row>
+    <row r="12" ht="31.5" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>TASK-011</t>
@@ -1741,8 +2050,8 @@
       <c r="F12" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="9" t="inlineStr"/>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="9" t="n"/>
       <c r="I12" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -1753,11 +2062,11 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K12" s="9" t="inlineStr"/>
-      <c r="L12" s="3" t="inlineStr"/>
-      <c r="M12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
+      <c r="K12" s="9" t="n"/>
+      <c r="L12" s="3" t="n"/>
+      <c r="M12" s="3" t="n"/>
+    </row>
+    <row r="13" ht="31.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>TASK-012</t>
@@ -1786,8 +2095,8 @@
       <c r="F13" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="9" t="inlineStr"/>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="9" t="n"/>
       <c r="I13" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -1798,9 +2107,9 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K13" s="9" t="inlineStr"/>
-      <c r="L13" s="3" t="inlineStr"/>
-      <c r="M13" s="3" t="inlineStr"/>
+      <c r="K13" s="9" t="n"/>
+      <c r="L13" s="3" t="n"/>
+      <c r="M13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1831,8 +2140,8 @@
       <c r="F14" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="9" t="inlineStr"/>
+      <c r="G14" s="3" t="n"/>
+      <c r="H14" s="9" t="n"/>
       <c r="I14" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -1843,11 +2152,11 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K14" s="9" t="inlineStr"/>
-      <c r="L14" s="3" t="inlineStr"/>
-      <c r="M14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15">
+      <c r="K14" s="9" t="n"/>
+      <c r="L14" s="3" t="n"/>
+      <c r="M14" s="3" t="n"/>
+    </row>
+    <row r="15" ht="31.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>TASK-014</t>
@@ -1876,8 +2185,8 @@
       <c r="F15" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="9" t="inlineStr"/>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="9" t="n"/>
       <c r="I15" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -1888,11 +2197,11 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K15" s="9" t="inlineStr"/>
-      <c r="L15" s="3" t="inlineStr"/>
-      <c r="M15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16">
+      <c r="K15" s="9" t="n"/>
+      <c r="L15" s="3" t="n"/>
+      <c r="M15" s="3" t="n"/>
+    </row>
+    <row r="16" ht="31.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>TASK-015</t>
@@ -1921,8 +2230,8 @@
       <c r="F16" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="3" t="inlineStr"/>
-      <c r="H16" s="9" t="inlineStr"/>
+      <c r="G16" s="3" t="n"/>
+      <c r="H16" s="9" t="n"/>
       <c r="I16" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -1933,11 +2242,11 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K16" s="9" t="inlineStr"/>
-      <c r="L16" s="3" t="inlineStr"/>
-      <c r="M16" s="3" t="inlineStr"/>
-    </row>
-    <row r="17">
+      <c r="K16" s="9" t="n"/>
+      <c r="L16" s="3" t="n"/>
+      <c r="M16" s="3" t="n"/>
+    </row>
+    <row r="17" ht="31.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>TASK-016</t>
@@ -1966,8 +2275,8 @@
       <c r="F17" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G17" s="3" t="inlineStr"/>
-      <c r="H17" s="9" t="inlineStr"/>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="9" t="n"/>
       <c r="I17" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -1978,11 +2287,11 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K17" s="9" t="inlineStr"/>
-      <c r="L17" s="3" t="inlineStr"/>
-      <c r="M17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18">
+      <c r="K17" s="9" t="n"/>
+      <c r="L17" s="3" t="n"/>
+      <c r="M17" s="3" t="n"/>
+    </row>
+    <row r="18" ht="47.25" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>TASK-017</t>
@@ -2047,7 +2356,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="47.25" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>TASK-018</t>
@@ -2112,7 +2421,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="31.5" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t>TASK-019</t>
@@ -2177,7 +2486,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="47.25" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t>TASK-020</t>
@@ -2242,7 +2551,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="31.5" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>TASK-021</t>
@@ -2271,8 +2580,8 @@
       <c r="F22" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="3" t="inlineStr"/>
-      <c r="H22" s="9" t="inlineStr"/>
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="9" t="n"/>
       <c r="I22" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -2283,11 +2592,11 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K22" s="9" t="inlineStr"/>
-      <c r="L22" s="3" t="inlineStr"/>
-      <c r="M22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23">
+      <c r="K22" s="9" t="n"/>
+      <c r="L22" s="3" t="n"/>
+      <c r="M22" s="3" t="n"/>
+    </row>
+    <row r="23" ht="47.25" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
           <t>TASK-022</t>
@@ -2381,8 +2690,8 @@
       <c r="F24" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G24" s="3" t="inlineStr"/>
-      <c r="H24" s="9" t="inlineStr"/>
+      <c r="G24" s="3" t="n"/>
+      <c r="H24" s="9" t="n"/>
       <c r="I24" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -2393,9 +2702,9 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K24" s="9" t="inlineStr"/>
-      <c r="L24" s="3" t="inlineStr"/>
-      <c r="M24" s="3" t="inlineStr"/>
+      <c r="K24" s="9" t="n"/>
+      <c r="L24" s="3" t="n"/>
+      <c r="M24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -2426,8 +2735,8 @@
       <c r="F25" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="9" t="inlineStr"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="9" t="n"/>
       <c r="I25" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -2438,11 +2747,11 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K25" s="9" t="inlineStr"/>
-      <c r="L25" s="3" t="inlineStr"/>
-      <c r="M25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26">
+      <c r="K25" s="9" t="n"/>
+      <c r="L25" s="3" t="n"/>
+      <c r="M25" s="3" t="n"/>
+    </row>
+    <row r="26" ht="63" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
           <t>TASK-025</t>
@@ -2536,8 +2845,8 @@
       <c r="F27" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="3" t="inlineStr"/>
-      <c r="H27" s="9" t="inlineStr"/>
+      <c r="G27" s="3" t="n"/>
+      <c r="H27" s="9" t="n"/>
       <c r="I27" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -2548,11 +2857,11 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K27" s="9" t="inlineStr"/>
-      <c r="L27" s="3" t="inlineStr"/>
-      <c r="M27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28">
+      <c r="K27" s="9" t="n"/>
+      <c r="L27" s="3" t="n"/>
+      <c r="M27" s="3" t="n"/>
+    </row>
+    <row r="28" ht="31.5" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
         <is>
           <t>TASK-027</t>
@@ -2617,7 +2926,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="47.25" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
           <t>TASK-028</t>
@@ -2682,7 +2991,7 @@
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="63" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
         <is>
           <t>TASK-029</t>
@@ -2747,7 +3056,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="47.25" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t>TASK-030</t>
@@ -2812,7 +3121,7 @@
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="78.75" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
         <is>
           <t>TASK-031</t>
@@ -2877,7 +3186,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="63" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
           <t>TASK-032</t>
@@ -2942,7 +3251,7 @@
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="63" customHeight="1">
       <c r="A34" s="3" t="inlineStr">
         <is>
           <t>TASK-033</t>
@@ -3007,7 +3316,7 @@
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="47.25" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>TASK-034</t>
@@ -3072,7 +3381,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="47.25" customHeight="1">
       <c r="A36" s="3" t="inlineStr">
         <is>
           <t>TASK-035</t>
@@ -3166,8 +3475,8 @@
       <c r="F37" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G37" s="3" t="inlineStr"/>
-      <c r="H37" s="9" t="inlineStr"/>
+      <c r="G37" s="3" t="n"/>
+      <c r="H37" s="9" t="n"/>
       <c r="I37" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -3178,9 +3487,9 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K37" s="9" t="inlineStr"/>
-      <c r="L37" s="3" t="inlineStr"/>
-      <c r="M37" s="3" t="inlineStr"/>
+      <c r="K37" s="9" t="n"/>
+      <c r="L37" s="3" t="n"/>
+      <c r="M37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -3211,8 +3520,8 @@
       <c r="F38" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="3" t="inlineStr"/>
-      <c r="H38" s="9" t="inlineStr"/>
+      <c r="G38" s="3" t="n"/>
+      <c r="H38" s="9" t="n"/>
       <c r="I38" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -3223,11 +3532,11 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K38" s="9" t="inlineStr"/>
-      <c r="L38" s="3" t="inlineStr"/>
-      <c r="M38" s="3" t="inlineStr"/>
-    </row>
-    <row r="39">
+      <c r="K38" s="9" t="n"/>
+      <c r="L38" s="3" t="n"/>
+      <c r="M38" s="3" t="n"/>
+    </row>
+    <row r="39" ht="31.5" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
         <is>
           <t>TASK-038</t>
@@ -3256,8 +3565,8 @@
       <c r="F39" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G39" s="3" t="inlineStr"/>
-      <c r="H39" s="9" t="inlineStr"/>
+      <c r="G39" s="3" t="n"/>
+      <c r="H39" s="9" t="n"/>
       <c r="I39" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -3268,11 +3577,11 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K39" s="9" t="inlineStr"/>
-      <c r="L39" s="3" t="inlineStr"/>
-      <c r="M39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40">
+      <c r="K39" s="9" t="n"/>
+      <c r="L39" s="3" t="n"/>
+      <c r="M39" s="3" t="n"/>
+    </row>
+    <row r="40" ht="31.5" customHeight="1">
       <c r="A40" s="3" t="inlineStr">
         <is>
           <t>TASK-039</t>
@@ -3301,8 +3610,8 @@
       <c r="F40" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G40" s="3" t="inlineStr"/>
-      <c r="H40" s="9" t="inlineStr"/>
+      <c r="G40" s="3" t="n"/>
+      <c r="H40" s="9" t="n"/>
       <c r="I40" s="3" t="inlineStr">
         <is>
           <t>TODO0314 section 5</t>
@@ -3313,9 +3622,9 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="K40" s="9" t="inlineStr"/>
-      <c r="L40" s="3" t="inlineStr"/>
-      <c r="M40" s="3" t="inlineStr"/>
+      <c r="K40" s="9" t="n"/>
+      <c r="L40" s="3" t="n"/>
+      <c r="M40" s="3" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:M40"/>
@@ -3323,7 +3632,7 @@
     <dataValidation sqref="E2:E40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not Started,In Progress,Blocked,Done"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+    <dataValidation sqref="F2:F40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
@@ -3338,8 +3647,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -3392,10 +3701,10 @@
           <t>??????</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr"/>
-      <c r="D2" s="3" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
-      <c r="F2" s="3" t="inlineStr"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3694,14 +4003,58 @@
           <t>[AUTO] Commit recorded: main @ d320697</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>Continue task updates and prepare push.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-03-25 00:09:02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ 0012f38</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-03-28 21:35:01</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ 367b31a</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
         <is>
           <t>git-hook</t>
         </is>
@@ -3719,17 +4072,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="3" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="6" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -3811,9 +4160,9 @@
           <t>Top UX + Admin UX</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr"/>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="3" t="inlineStr"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
       <c r="I2" s="3" t="inlineStr">
         <is>
           <t>c85c8b0</t>
@@ -3842,8 +4191,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -4419,7 +4768,81 @@
           <t>https://github.com/dan40912/prayer-coin.git</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-03-25 00:09:02</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0012f38</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>(no tag)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>feat: improve SEO metadata, footer spacing, and customer image upload flow</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/prayer-coin.git</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-03-28 21:35:01</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>367b31a</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>(no tag)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>release: v2.0.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/prayer-coin.git</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: update progress tracker workbook
</commit_message>
<xml_diff>
--- a/output/spreadsheet/startpray-progress-tracker.xlsx
+++ b/output/spreadsheet/startpray-progress-tracker.xlsx
@@ -599,7 +599,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>367b31a</t>
+          <t>0091916</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>(no tag)</t>
+          <t>v2</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-03-28 21:35:01</t>
+          <t>2026-03-30 01:24:29</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4047,14 +4047,36 @@
           <t>[AUTO] Commit recorded: main @ 367b31a</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>Continue task updates and prepare push.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-03-30 01:24:29</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ 0091916</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
         <is>
           <t>git-hook</t>
         </is>
@@ -4191,7 +4213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4842,7 +4864,44 @@
           <t>https://github.com/dan40912/prayer-coin.git</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-03-30 01:24:29</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>0091916</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>feat: finalize admin editors/player updates and add prod migration bundle</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/prayer-coin.git</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update auth sessions and customer portal flow
</commit_message>
<xml_diff>
--- a/output/spreadsheet/startpray-progress-tracker.xlsx
+++ b/output/spreadsheet/startpray-progress-tracker.xlsx
@@ -599,7 +599,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>0091916</t>
+          <t>8eeb610</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-03-30 01:24:29</t>
+          <t>2026-04-02 23:17:07</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4069,14 +4069,80 @@
           <t>[AUTO] Commit recorded: main @ 0091916</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>Continue task updates and prepare push.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-03-30 01:24:58</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ 71c12b7</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03-31 00:16:22</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ 6ea34be</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-02 23:17:07</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ 8eeb610</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
         <is>
           <t>git-hook</t>
         </is>
@@ -4213,7 +4279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4901,7 +4967,118 @@
           <t>https://github.com/dan40912/prayer-coin.git</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-03-30 01:24:58</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>71c12b7</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>chore: update progress tracker workbook</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/prayer-coin.git</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-03-31 00:16:22</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>6ea34be</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Fix global player replay diagnostics and loop behavior</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/prayer-coin.git</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04-02 23:17:07</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>8eeb610</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Remove legacy wireframe assets</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/prayer-coin.git</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add global prayer room experience and prayer seed tooling
</commit_message>
<xml_diff>
--- a/output/spreadsheet/startpray-progress-tracker.xlsx
+++ b/output/spreadsheet/startpray-progress-tracker.xlsx
@@ -599,7 +599,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>8eeb610</t>
+          <t>ce22e58</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-04-02 23:17:07</t>
+          <t>2026-04-26 13:09:29</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4135,14 +4135,58 @@
           <t>[AUTO] Commit recorded: main @ 8eeb610</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>Continue task updates and prepare push.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-04-26 12:57:49</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ 7d71f48</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-04-26 13:09:29</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ ce22e58</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
         <is>
           <t>git-hook</t>
         </is>
@@ -4279,7 +4323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5078,7 +5122,81 @@
           <t>https://github.com/dan40912/prayer-coin.git</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-26 12:57:49</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>7d71f48</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Add overcomer story media and SEO updates</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/prayer-coin.git</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-04-26 13:09:29</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ce22e58</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Improve overcomer story recording modal</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/prayer-coin.git</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Start Pray docs and public UI
</commit_message>
<xml_diff>
--- a/output/spreadsheet/startpray-progress-tracker.xlsx
+++ b/output/spreadsheet/startpray-progress-tracker.xlsx
@@ -599,7 +599,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>ce22e58</t>
+          <t>dee4b64</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-04-26 13:09:29</t>
+          <t>2026-05-10 19:36:25</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4179,14 +4179,102 @@
           <t>[AUTO] Commit recorded: main @ ce22e58</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>Continue task updates and prepare push.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-05 00:56:10</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ d8dfbe6</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-09 20:01:08</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ b034091</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-10 19:36:02</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ c3a856b</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-10 19:36:25</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ dee4b64</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
         <is>
           <t>git-hook</t>
         </is>
@@ -4323,7 +4411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5196,7 +5284,155 @@
           <t>https://github.com/dan40912/prayer-coin.git</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-05 00:56:10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>d8dfbe6</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Add global prayer room experience and prayer seed tooling</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/prayer-coin.git</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-09 20:01:08</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>b034091</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Improve global prayer room map experience</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/prayer-coin.git</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-10 19:36:02</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>c3a856b</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Update Start Pray docs and public UI</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-10 19:36:25</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>dee4b64</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Update Start Pray docs and public UI</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>